<commit_message>
added bug-report-log.md modified:   test_docs/BUG_001B.md modified:   test_docs/test-cases-navigation-ui.xlsx modified:   test_docs/test-plan-v1.0.md modified:   test_docs/test-plan-v2.0.md modified:   test_docs/test-summary-v1.0.md
</commit_message>
<xml_diff>
--- a/test_docs/test-cases-navigation-ui.xlsx
+++ b/test_docs/test-cases-navigation-ui.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Portfolio\e-commerce_app\test_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA4D7606-030D-4CE8-AE7F-5D3B7E7AC9F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCAAB16-F694-4393-A555-D23F559F4DE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{8DC2A5E5-04F7-4C0F-86D2-4C7937B2014E}"/>
   </bookViews>
@@ -450,21 +450,21 @@
 4.The menu can be closed manually by clicking the cross icon </t>
   </si>
   <si>
+    <t>N/A</t>
+  </si>
+  <si>
     <t>1. The menu opens when hamburger is clicked
 2.The hamburger doesn't turn into a cross
 3.A cross appears on the menu toggle window itself, below the hamburger
-4.The menu doesn't automatically closes after selecting a page
+4.The menu doesn't automatically close after selecting a page
 5.The menu closes after clicking the hamburger or the cross icon</t>
-  </si>
-  <si>
-    <t>N/A</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -494,12 +494,6 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <color rgb="FF0F1115"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color rgb="FF0F1115"/>
       <name val="Segoe UI"/>
@@ -1215,13 +1209,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="116">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1231,25 +1223,18 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1262,16 +1247,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1304,9 +1286,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1315,9 +1294,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1330,16 +1306,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1357,16 +1330,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment textRotation="45"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1375,45 +1348,41 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="45" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="44" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment textRotation="45"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1422,13 +1391,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2432,269 +2401,262 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="H1" s="82"/>
-      <c r="I1" s="85"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="20"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="13"/>
+      <c r="L1" s="14"/>
     </row>
     <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="5" t="s">
+      <c r="B2" s="4"/>
+      <c r="C2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="87" t="s">
+      <c r="E2" s="72" t="s">
         <v>25</v>
       </c>
-      <c r="H2" s="89"/>
-      <c r="I2" s="84"/>
-      <c r="J2" s="21"/>
-      <c r="K2" s="22"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="17"/>
+      <c r="H2" s="74"/>
+      <c r="I2" s="70"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="12"/>
     </row>
     <row r="3" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="2" t="s">
+      <c r="B3" s="5"/>
+      <c r="C3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="88">
+      <c r="E3" s="73">
         <v>46303</v>
       </c>
-      <c r="G3" s="62"/>
-      <c r="H3" s="83"/>
-      <c r="I3" s="86"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="23"/>
-      <c r="L3" s="23"/>
-      <c r="M3" s="17"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="69"/>
+      <c r="I3" s="71"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11"/>
+      <c r="M3" s="12"/>
     </row>
     <row r="4" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="4" t="s">
+      <c r="B4" s="6"/>
+      <c r="C4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="90" t="s">
+      <c r="E4" s="75" t="s">
         <v>42</v>
       </c>
-      <c r="F4" s="1"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="81"/>
-      <c r="J4" s="63"/>
-      <c r="K4" s="24"/>
-      <c r="L4" s="25"/>
+      <c r="I4" s="68"/>
+      <c r="J4" s="50"/>
+      <c r="L4" s="14"/>
     </row>
     <row r="5" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="J5" s="26"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="16"/>
+      <c r="J5" s="17"/>
+      <c r="L5" s="11"/>
     </row>
     <row r="6" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="38" t="s">
+      <c r="A6" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="38" t="s">
+      <c r="C6" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="38" t="s">
+      <c r="D6" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="38" t="s">
+      <c r="E6" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="39" t="s">
+      <c r="F6" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="39" t="s">
+      <c r="G6" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="40" t="s">
+      <c r="H6" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="I6" s="28" t="s">
+      <c r="I6" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="J6" s="41" t="s">
+      <c r="J6" s="31" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="131" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="42" t="s">
+      <c r="A7" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="43" t="s">
+      <c r="B7" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="44" t="s">
+      <c r="C7" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="45" t="s">
+      <c r="D7" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="46" t="s">
+      <c r="E7" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="46" t="s">
+      <c r="F7" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="G7" s="43" t="s">
+      <c r="G7" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="47" t="s">
+      <c r="H7" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="I7" s="47"/>
-      <c r="J7" s="48" t="s">
+      <c r="I7" s="37"/>
+      <c r="J7" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="K7" s="37"/>
+      <c r="K7" s="27"/>
     </row>
     <row r="8" spans="1:16" ht="131" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="49" t="s">
+      <c r="A8" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="50" t="s">
+      <c r="B8" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="33" t="s">
+      <c r="D8" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="32" t="s">
+      <c r="E8" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="32" t="s">
+      <c r="F8" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="G8" s="50" t="s">
+      <c r="G8" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="H8" s="29" t="s">
+      <c r="H8" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="I8" s="27"/>
-      <c r="J8" s="51" t="s">
+      <c r="I8" s="18"/>
+      <c r="J8" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
     </row>
     <row r="9" spans="1:16" ht="131" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="49" t="s">
+      <c r="A9" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="33" t="s">
+      <c r="D9" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="32" t="s">
+      <c r="E9" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="34" t="s">
+      <c r="F9" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="G9" s="34" t="s">
+      <c r="G9" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="H9" s="29" t="s">
+      <c r="H9" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="I9" s="27"/>
-      <c r="J9" s="51" t="s">
+      <c r="I9" s="18"/>
+      <c r="J9" s="40" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="131" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="49" t="s">
+      <c r="A10" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="27" t="s">
+      <c r="C10" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="33" t="s">
+      <c r="D10" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="32" t="s">
+      <c r="E10" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="60" t="s">
+      <c r="F10" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="G10" s="34" t="s">
+      <c r="G10" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="H10" s="29" t="s">
+      <c r="H10" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="I10" s="27"/>
-      <c r="J10" s="51" t="s">
+      <c r="I10" s="18"/>
+      <c r="J10" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="P10" s="57"/>
+      <c r="P10" s="45"/>
     </row>
     <row r="11" spans="1:16" ht="131" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="52" t="s">
+      <c r="A11" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="31" t="s">
+      <c r="B11" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="53" t="s">
+      <c r="C11" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="54" t="s">
+      <c r="D11" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="31" t="s">
+      <c r="E11" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="F11" s="61" t="s">
+      <c r="F11" s="48" t="s">
         <v>40</v>
       </c>
-      <c r="G11" s="58" t="s">
+      <c r="G11" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="H11" s="55" t="s">
+      <c r="H11" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="I11" s="53"/>
-      <c r="J11" s="56" t="s">
+      <c r="I11" s="42"/>
+      <c r="J11" s="44" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="F12" s="59"/>
+      <c r="F12" s="47"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2720,213 +2682,213 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="E1" s="68"/>
+      <c r="E1" s="55"/>
     </row>
     <row r="2" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="5" t="s">
+      <c r="B2" s="4"/>
+      <c r="C2" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="D2" s="94" t="s">
+      <c r="D2" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="97" t="s">
+      <c r="E2" s="80" t="s">
         <v>25</v>
       </c>
-      <c r="H2" s="93"/>
+      <c r="H2" s="70"/>
     </row>
     <row r="3" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="2" t="s">
+      <c r="B3" s="5"/>
+      <c r="C3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="95" t="s">
+      <c r="D3" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="98">
+      <c r="E3" s="81">
         <v>46303</v>
       </c>
-      <c r="H3" s="92"/>
+      <c r="H3" s="71"/>
     </row>
     <row r="4" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="4" t="s">
+      <c r="B4" s="6"/>
+      <c r="C4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="35" t="s">
+      <c r="D4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="96" t="s">
+      <c r="E4" s="79" t="s">
         <v>42</v>
       </c>
-      <c r="H4" s="92"/>
+      <c r="H4" s="71"/>
     </row>
     <row r="5" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="6" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="69" t="s">
+      <c r="A6" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="70" t="s">
+      <c r="B6" s="57" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="70" t="s">
+      <c r="C6" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="70" t="s">
+      <c r="D6" s="57" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="70" t="s">
+      <c r="E6" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="71" t="s">
+      <c r="F6" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="71" t="s">
+      <c r="G6" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="28" t="s">
+      <c r="H6" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="I6" s="28" t="s">
+      <c r="I6" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="J6" s="72" t="s">
+      <c r="J6" s="59" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="99" t="s">
+      <c r="A7" s="82" t="s">
         <v>44</v>
       </c>
-      <c r="B7" s="43" t="s">
+      <c r="B7" s="33" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="73" t="s">
+      <c r="C7" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="43" t="s">
+      <c r="D7" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="E7" s="46" t="s">
+      <c r="E7" s="36" t="s">
         <v>51</v>
       </c>
-      <c r="F7" s="109" t="s">
-        <v>86</v>
-      </c>
-      <c r="G7" s="74" t="s">
+      <c r="F7" s="92" t="s">
+        <v>85</v>
+      </c>
+      <c r="G7" s="61" t="s">
         <v>45</v>
       </c>
-      <c r="H7" s="47" t="s">
+      <c r="H7" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="I7" s="47"/>
-      <c r="J7" s="51" t="s">
+      <c r="I7" s="37"/>
+      <c r="J7" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="L7" s="91"/>
-      <c r="M7" s="77"/>
+      <c r="L7" s="76"/>
+      <c r="M7" s="64"/>
     </row>
     <row r="8" spans="1:13" ht="87.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A8" s="100" t="s">
+      <c r="A8" s="83" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="50" t="s">
+      <c r="B8" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="75" t="s">
+      <c r="C8" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="76" t="s">
+      <c r="D8" s="63" t="s">
         <v>53</v>
       </c>
-      <c r="E8" s="32" t="s">
+      <c r="E8" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="F8" s="109" t="s">
-        <v>86</v>
-      </c>
-      <c r="G8" s="78" t="s">
+      <c r="F8" s="92" t="s">
+        <v>85</v>
+      </c>
+      <c r="G8" s="65" t="s">
         <v>45</v>
       </c>
-      <c r="H8" s="27" t="s">
+      <c r="H8" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="I8" s="27"/>
-      <c r="J8" s="51" t="s">
+      <c r="I8" s="18"/>
+      <c r="J8" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="L8" s="91"/>
+      <c r="L8" s="76"/>
     </row>
     <row r="9" spans="1:13" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="100" t="s">
+      <c r="A9" s="83" t="s">
         <v>49</v>
       </c>
-      <c r="B9" s="50" t="s">
+      <c r="B9" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C9" s="75" t="s">
+      <c r="C9" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="E9" s="32" t="s">
+      <c r="E9" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="F9" s="109" t="s">
-        <v>86</v>
-      </c>
-      <c r="G9" s="9" t="s">
+      <c r="F9" s="92" t="s">
+        <v>85</v>
+      </c>
+      <c r="G9" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="H9" s="27" t="s">
+      <c r="H9" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="I9" s="27"/>
-      <c r="J9" s="51" t="s">
+      <c r="I9" s="18"/>
+      <c r="J9" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="L9" s="91"/>
+      <c r="L9" s="76"/>
     </row>
     <row r="10" spans="1:13" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="101" t="s">
+      <c r="A10" s="84" t="s">
         <v>50</v>
       </c>
-      <c r="B10" s="80" t="s">
+      <c r="B10" s="67" t="s">
         <v>47</v>
       </c>
-      <c r="C10" s="79" t="s">
+      <c r="C10" s="66" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="80" t="s">
+      <c r="D10" s="67" t="s">
         <v>52</v>
       </c>
-      <c r="E10" s="31" t="s">
+      <c r="E10" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="F10" s="109" t="s">
-        <v>86</v>
-      </c>
-      <c r="G10" s="31" t="s">
+      <c r="F10" s="92" t="s">
+        <v>85</v>
+      </c>
+      <c r="G10" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="H10" s="53" t="s">
+      <c r="H10" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="I10" s="53"/>
-      <c r="J10" s="56" t="s">
+      <c r="I10" s="42"/>
+      <c r="J10" s="44" t="s">
         <v>25</v>
       </c>
-      <c r="L10" s="91"/>
+      <c r="L10" s="76"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2952,163 +2914,163 @@
   <sheetData>
     <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="5" t="s">
+      <c r="B2" s="4"/>
+      <c r="C2" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D2" s="94" t="s">
+      <c r="D2" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="97" t="s">
+      <c r="E2" s="80" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="2" t="s">
+      <c r="B3" s="5"/>
+      <c r="C3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="95" t="s">
+      <c r="D3" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="98">
+      <c r="E3" s="81">
         <v>46303</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="4" t="s">
+      <c r="B4" s="6"/>
+      <c r="C4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="35" t="s">
+      <c r="D4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="96" t="s">
+      <c r="E4" s="79" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="6" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="40" t="s">
+      <c r="A6" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="64" t="s">
+      <c r="B6" s="51" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="65" t="s">
+      <c r="C6" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="65" t="s">
+      <c r="D6" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="65" t="s">
+      <c r="E6" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="66" t="s">
+      <c r="F6" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="40" t="s">
+      <c r="G6" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="H6" s="40" t="s">
+      <c r="H6" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="I6" s="67" t="s">
+      <c r="I6" s="54" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="103" t="s">
+      <c r="A7" s="86" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="43" t="s">
+      <c r="B7" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="C7" s="73" t="s">
+      <c r="C7" s="60" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="36" t="s">
         <v>65</v>
       </c>
-      <c r="E7" s="46" t="s">
+      <c r="E7" s="36" t="s">
         <v>63</v>
       </c>
-      <c r="F7" s="43" t="s">
+      <c r="F7" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="G7" s="47" t="s">
+      <c r="G7" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="H7" s="47"/>
-      <c r="I7" s="48" t="s">
+      <c r="H7" s="37"/>
+      <c r="I7" s="38" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="104" t="s">
+      <c r="A8" s="87" t="s">
         <v>68</v>
       </c>
-      <c r="B8" s="50" t="s">
+      <c r="B8" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D8" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="E8" s="32" t="s">
+      <c r="E8" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="F8" s="32" t="s">
+      <c r="F8" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="G8" s="27" t="s">
+      <c r="G8" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="H8" s="27"/>
-      <c r="I8" s="51" t="s">
+      <c r="H8" s="18"/>
+      <c r="I8" s="40" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="76" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="52" t="s">
+      <c r="A9" s="41" t="s">
         <v>71</v>
       </c>
-      <c r="B9" s="80" t="s">
+      <c r="B9" s="67" t="s">
         <v>72</v>
       </c>
-      <c r="C9" s="53" t="s">
+      <c r="C9" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="D9" s="31" t="s">
+      <c r="D9" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="E9" s="105" t="s">
+      <c r="E9" s="88" t="s">
         <v>74</v>
       </c>
-      <c r="F9" s="80" t="s">
+      <c r="F9" s="67" t="s">
         <v>75</v>
       </c>
-      <c r="G9" s="53" t="s">
+      <c r="G9" s="42" t="s">
         <v>64</v>
       </c>
-      <c r="H9" s="53"/>
-      <c r="I9" s="56" t="s">
+      <c r="H9" s="42"/>
+      <c r="I9" s="44" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C11" s="102"/>
+      <c r="C11" s="85"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3133,107 +3095,107 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C1" s="68"/>
+      <c r="C1" s="55"/>
     </row>
     <row r="2" spans="1:9" ht="16" x14ac:dyDescent="0.45">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="107"/>
-      <c r="C2" s="108" t="s">
+      <c r="B2" s="90"/>
+      <c r="C2" s="91" t="s">
         <v>78</v>
       </c>
-      <c r="D2" s="106" t="s">
+      <c r="D2" s="89" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="97" t="s">
+      <c r="E2" s="80" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="2" t="s">
+      <c r="B3" s="5"/>
+      <c r="C3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="95" t="s">
+      <c r="D3" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="98">
+      <c r="E3" s="81">
         <v>46303</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="4" t="s">
+      <c r="B4" s="6"/>
+      <c r="C4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="35" t="s">
+      <c r="D4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="96" t="s">
+      <c r="E4" s="79" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="6" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="69" t="s">
+      <c r="B6" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="70" t="s">
+      <c r="C6" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="70" t="s">
+      <c r="D6" s="57" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="70" t="s">
+      <c r="E6" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="71" t="s">
+      <c r="F6" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="28" t="s">
+      <c r="G6" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="H6" s="28" t="s">
+      <c r="H6" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="I6" s="72" t="s">
+      <c r="I6" s="59" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="208.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A7" s="110" t="s">
+      <c r="A7" s="93" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="111" t="s">
+      <c r="B7" s="94" t="s">
         <v>80</v>
       </c>
-      <c r="C7" s="112" t="s">
+      <c r="C7" s="95" t="s">
         <v>79</v>
       </c>
-      <c r="D7" s="113" t="s">
+      <c r="D7" s="96" t="s">
         <v>81</v>
       </c>
-      <c r="E7" s="113" t="s">
+      <c r="E7" s="96" t="s">
         <v>82</v>
       </c>
-      <c r="F7" s="113" t="s">
+      <c r="F7" s="96" t="s">
         <v>84</v>
       </c>
-      <c r="G7" s="114" t="s">
-        <v>85</v>
-      </c>
-      <c r="H7" s="36"/>
-      <c r="I7" s="115" t="s">
+      <c r="G7" s="97" t="s">
+        <v>86</v>
+      </c>
+      <c r="H7" s="26"/>
+      <c r="I7" s="98" t="s">
         <v>83</v>
       </c>
     </row>

</xml_diff>